<commit_message>
Import hardware parts and inventory from Excel (Screw, Washer, Grommet, Spacer, Bolt, Nut, Thimble)
</commit_message>
<xml_diff>
--- a/Category wise.xlsx
+++ b/Category wise.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc3138b539fcc989/Desktop/SUPERSYSTEMS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_91E47C5E47EDDA7985BA9672C209C726427CE330" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{629042FB-6091-472B-B884-6B5DBFEE29EF}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_91E47C5E47EDDA7985BA9672C209C726427CE330" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE526706-C19A-448F-987F-F9372D62617D}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="929" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="929" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mosfet" sheetId="1" r:id="rId1"/>
@@ -9808,6 +9808,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>